<commit_message>
Rewrite Sugar News 2026-09-13 summaries
</commit_message>
<xml_diff>
--- a/reports/2026/09/Sugar News 2026-09-13.xlsx
+++ b/reports/2026/09/Sugar News 2026-09-13.xlsx
@@ -505,7 +505,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="164.25" customHeight="1" s="2">
+    <row r="2" ht="180" customHeight="1" s="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -513,16 +513,16 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>印度政府披露糖厂运行和压榨安排，披露70 crore、Rs 70。印度糖厂运行信息需要落实到开榨、停产、压榨量或原料供应方向后判断阶段性供应。来源：The Times of India（https://timesofindia.indiatimes.com/city/patna/bihar-govt-sweetens-deal-for-new-sugar-mills-with-rs-70-crore-grant-over-5-years/articleshow/134143727.cms）。影响：利空糖价</t>
+          <t>印度比哈尔邦政府在《比哈尔甘蔗产业投资促进政策2026》中规定，新建糖厂最低压榨能力为3500 TCD，每座厂投产后5年合计可获70 crore卢比补贴，现有糖厂扩产1000 TCD可获15 crore卢比补贴。该政策降低比哈尔邦新建和扩建糖厂成本，项目落地后会提高当地甘蔗压榨能力和食糖产能，增加中期供应预期。来源：The Times of India（https://timesofindia.indiatimes.com/city/patna/bihar-govt-sweetens-deal-for-new-sugar-mills-with-rs-70-crore-grant-over-5-years/articleshow/134143727.cms）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>利空：糖厂运行、压榨能力或原料供应改善会提高食糖生产节奏，增加阶段性供应。</t>
+          <t>利空：比哈尔邦补贴新建和扩建糖厂会降低产能投资成本，项目落地后增加甘蔗压榨能力和中期食糖供应预期。</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="116.4" customHeight="1" s="2">
+    <row r="3" ht="169.2" customHeight="1" s="2">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>泰国</t>
@@ -530,16 +530,16 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>泰国糖业相关机构公布糖产量，糖产量下降17%。糖产量下降会减少当期新增可售糖源，收紧供应端并支撑糖价。来源：ukragroconsult.com（https://ukragroconsult.com/en/news/thailands-sugar-production-may-fall-by-at-least-17/）。影响：利多糖价</t>
+          <t>周末延续消息：泰国制糖商公司预计泰国2026/27榨季糖产量可能至少下降17%至低于1000万吨，低于上一榨季1200万吨；东北部约占全国食糖产量45%，今年降雨偏少且木薯价格较高可能挤占甘蔗面积。泰国是全球第二大食糖出口国，产量下修会减少可出口糖供应并收紧国际贸易流通量，对原糖价格形成支撑。来源：ukragroconsult.com（https://ukragroconsult.com/en/news/thailands-sugar-production-may-fall-by-at-least-17/）。影响：利多糖价</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>利多：糖产量下降会减少当期新增可售糖源，收紧供应端并支撑糖价。</t>
+          <t>利多：泰国糖产量下修会减少全球第二大出口国的可出口糖供应，收紧国际贸易流通量并支撑原糖价格。</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="180" customHeight="1" s="2">
+    <row r="4" ht="134.55" customHeight="1" s="2">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>泰国</t>
@@ -547,7 +547,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Open-Meteo预报显示（2026-09-14至2026-09-20），泰国东北部（呵叻、孔敬、乌隆他尼、猜也蓬）；北部（那空沙旺、甘烹碧、素可泰、彭世洛）；中部及西部（北碧、华富里、素攀武里、猜纳）；东部（沙缴、春武里）等主要甘蔗产区存在降雨预报，实际可用预报期为7日，累计预测降雨较高的监测点包括彭世洛约137.2mm、甘烹碧约134.2mm、素攀武里约124.2mm。当前处于甘蔗生长阶段，降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：Open-Meteo（https://api.open-meteo.com/v1/forecast）。影响：利空糖价</t>
+          <t>Open-Meteo预报显示，9月14日至20日泰国东北部、北部、中西部和东部主要甘蔗产区均有降雨，其中彭世洛、甘烹碧、素攀武里7日累计降雨分别约137.2mm、134.2mm、124.2mm。泰国甘蔗仍处生长期，上述降雨会补充土壤水分、改善墒情并提高后期甘蔗单产和食糖产量预期。来源：Open-Meteo（https://api.open-meteo.com/v1/forecast）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">

</xml_diff>